<commit_message>
feat(v1.6): 新增氣喘/濕疹評估分紅 (Peak flow/ACT/POEM, \$5/筆)
- 計算鏡射自費流感: 評估筆數從 60 人門檻扣除 + 每筆獨立給 \$5,
  進基礎分紅池 (時段當班所有人平分)
- Form 1 新增必填欄位「氣喘/濕疹評估筆數」(一位病人一次門診算 1 筆)
- 「分紅明細」新增 J 欄「評估筆數」(僅基礎分紅列填值)
- 月度結算區塊 4 加入評估筆數欄
- migrateDailyFormAddAssessment(): 既有部署一鍵在 Form 1 加欄位
- testCalculation 擴充至 10 個 case (全數通過模擬驗證)
- 單價參數/xlsx/DEPLOYMENT.md 對應更新
</commit_message>
<xml_diff>
--- a/clinic_bonus_template.xlsx
+++ b/clinic_bonus_template.xlsx
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -766,82 +766,89 @@
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>基礎分紅 = MAX(0, 看診 - 流感 - 60) × 5 + 流感 × 5（每位當班員工平均分）。</t>
+          <t>基礎分紅 = MAX(0, 看診 - 流感 - 評估 - 60) × 5 + 流感 × 5 + 評估 × 5。</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>值日生津貼 = 100 元（僅上午/下午、值日生一人）。</t>
+          <t>（評估 = Peak flow/ACT/POEM，一位病人一次算 1 筆；每位當班員工平均分）</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>代謝症候群：收案 100 元/筆、追蹤 20 元/筆，給該筆執行人員。</t>
+          <t>值日生津貼 = 100 元（僅上午/下午、值日生一人）。</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
+          <t>代謝症候群：收案 100 元/筆、追蹤 20 元/筆，給該筆執行人員。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
           <t>詳見 README.md 與 apps_script.gs。</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>六、分頁清單</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>1. 員工總表（唯一手動維護處）</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>2. 單價參數</t>
+          <t>1. 員工總表（唯一手動維護處）</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>3. Form回應_當班（Form 1 自動寫入）</t>
+          <t>2. 單價參數</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>4. Form回應_代謝（Form 2 自動寫入）</t>
+          <t>3. Form回應_當班（Form 1 自動寫入）</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>5. 分紅明細（Apps Script 自動 append，月結算來源）</t>
+          <t>4. Form回應_代謝（Form 2 自動寫入）</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
+          <t>5. 分紅明細（Apps Script 自動 append，月結算來源）</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
           <t>6. 月度結算（含 QUERY 公式，上傳 Sheets 後生效）</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="34">
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A39:E39"/>
     <mergeCell ref="A34:E34"/>
@@ -859,9 +866,9 @@
     <mergeCell ref="A27:E27"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A33:E33"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A32:E32"/>
     <mergeCell ref="A22:E22"/>
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A29:E29"/>
@@ -874,6 +881,7 @@
     <mergeCell ref="A19:E19"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A31:E31"/>
+    <mergeCell ref="A40:E40"/>
     <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1187,13 +1195,28 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
+          <t>氣喘/濕疹評估單價</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Peak flow/ACT/POEM 每筆 5 元，一位病人一次門診算 1 筆</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
           <t>值日生人數門檻</t>
         </is>
       </c>
-      <c r="B8" s="7" t="n">
+      <c r="B9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>（目前未使用，預留）</t>
         </is>
@@ -1224,7 +1247,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1236,7 +1259,8 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1286,6 +1310,11 @@
         </is>
       </c>
       <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>氣喘/濕疹評估筆數</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>備註</t>
         </is>
@@ -1364,7 +1393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1376,6 +1405,7 @@
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1422,6 +1452,11 @@
       <c r="I1" s="5" t="inlineStr">
         <is>
           <t>病歷號</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>評估筆數</t>
         </is>
       </c>
     </row>
@@ -1509,7 +1544,7 @@
         <v/>
       </c>
       <c r="L2">
-        <f>QUERY('Form回應_當班'!A:J,"SELECT B, C, H, I WHERE B &gt;= date '"&amp;TEXT(EOMONTH(TODAY(),-1)+1,"yyyy-MM-dd")&amp;"' AND B &lt;= date '"&amp;TEXT(EOMONTH(TODAY(),0),"yyyy-MM-dd")&amp;"' ORDER BY B, C LABEL B '日期', C '時段', H '看診人數', I '流感支數'", 1)</f>
+        <f>QUERY('Form回應_當班'!A:K,"SELECT B, C, H, I, J WHERE B &gt;= date '"&amp;TEXT(EOMONTH(TODAY(),-1)+1,"yyyy-MM-dd")&amp;"' AND B &lt;= date '"&amp;TEXT(EOMONTH(TODAY(),0),"yyyy-MM-dd")&amp;"' ORDER BY B, C LABEL B '日期', C '時段', H '看診人數', I '流感支數', J '評估筆數'", 1)</f>
         <v/>
       </c>
       <c r="V2" s="12" t="inlineStr">

</xml_diff>